<commit_message>
feat(ai): realistic feature generation, aligned training/serving pipeline, and promoted MC-GNN model
</commit_message>
<xml_diff>
--- a/datasets/kinfra_data.xlsx
+++ b/datasets/kinfra_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECTS\EcoLinkAI\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{867E6A04-7529-47F1-9615-CB80649837D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77E1C61D-A78B-41C1-AC43-536A8D39853D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="254">
   <si>
     <t>Company Name</t>
   </si>
@@ -191,12 +191,6 @@
     <t>https://www.ooppoottiltyre.com</t>
   </si>
   <si>
-    <t>KINFRA Industrial Park, Kannur</t>
-  </si>
-  <si>
-    <t>Kannur</t>
-  </si>
-  <si>
     <t>Kerala</t>
   </si>
   <si>
@@ -789,6 +783,9 @@
   </si>
   <si>
     <t>Sell to scrap dealer/other buyers in TN</t>
+  </si>
+  <si>
+    <t>KINFRA Industrial Park, Trivandrum</t>
   </si>
 </sst>
 </file>
@@ -1229,7 +1226,7 @@
         <v>170000</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -1252,7 +1249,7 @@
         <v>567000</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
@@ -1275,7 +1272,7 @@
         <v>440000</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -1543,478 +1540,478 @@
         <v>54</v>
       </c>
       <c r="I2" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="K2" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="M2" s="2">
         <v>82</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O2" s="2">
         <v>2004</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="G3" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>67</v>
-      </c>
       <c r="I3" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="K3" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="L3" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="M3" s="2">
         <v>75</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O3" s="2">
         <v>2010</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="I4" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="K4" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="M4" s="2">
         <v>88</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O4" s="2">
         <v>1998</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>83</v>
-      </c>
       <c r="I5" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="K5" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="L5" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="M5" s="2">
         <v>79</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O5" s="2">
         <v>2006</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>90</v>
-      </c>
       <c r="I6" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="K6" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="L6" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="M6" s="2">
         <v>71</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O6" s="2">
         <v>2012</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="H7" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G7" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>97</v>
-      </c>
       <c r="I7" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="K7" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="L7" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="M7" s="2">
         <v>84</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O7" s="2">
         <v>2001</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="G8" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>104</v>
-      </c>
       <c r="I8" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="K8" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="L8" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="M8" s="2">
         <v>91</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O8" s="2">
         <v>2015</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>26</v>
       </c>
       <c r="C9" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G9" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="I9" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="K9" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="L9" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="K9" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="M9" s="2">
         <v>73</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O9" s="2">
         <v>2009</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D10" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="H10" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="G10" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>117</v>
-      </c>
       <c r="I10" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="K10" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="L10" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="L10" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="M10" s="2">
         <v>80</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O10" s="2">
         <v>2003</v>
       </c>
       <c r="P10" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>30</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="G11" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>124</v>
-      </c>
       <c r="I11" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="K11" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="L11" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="M11" s="2">
         <v>93</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O11" s="2">
         <v>2017</v>
       </c>
       <c r="P11" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -2038,16 +2035,16 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>32</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>41</v>
@@ -2061,232 +2058,232 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>48</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>133</v>
-      </c>
       <c r="E3" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>150</v>
-      </c>
       <c r="E11" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -2312,39 +2309,39 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>32</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>155</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>48</v>
@@ -2356,277 +2353,277 @@
         <v>49</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="G4" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H5" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F6" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="I6" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>21</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F7" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H7" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="I7" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="G8" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="I8" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F9" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H9" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="I9" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F10" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H10" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="I10" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="G11" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="I11" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -2660,75 +2657,75 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>32</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>193</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>48</v>
@@ -2737,34 +2734,34 @@
         <v>10139.43</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G2" s="2">
         <v>73.45</v>
       </c>
       <c r="H2" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="I2" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>199</v>
-      </c>
       <c r="K2" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="L2" s="2">
         <v>17</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="N2" s="2">
         <v>48.39</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="P2" s="2">
         <v>5000</v>
@@ -2779,54 +2776,54 @@
         <v>9</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="3" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E3" s="2">
         <v>5088.3500000000004</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G3" s="2">
         <v>83.37</v>
       </c>
       <c r="H3" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="J3" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>205</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>207</v>
       </c>
       <c r="L3" s="2">
         <v>113.4</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="N3" s="2">
         <v>36.909999999999997</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="P3" s="2">
         <v>2500</v>
@@ -2841,54 +2838,54 @@
         <v>12</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E4" s="2">
         <v>3893.06</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G4" s="2">
         <v>95.11</v>
       </c>
       <c r="H4" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="J4" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>213</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>215</v>
       </c>
       <c r="L4" s="2">
         <v>110</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="N4" s="2">
         <v>77.959999999999994</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="P4" s="2">
         <v>4000</v>
@@ -2903,54 +2900,54 @@
         <v>15</v>
       </c>
       <c r="T4" s="2" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="5" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E5" s="2">
         <v>3471.83</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G5" s="2">
         <v>63.64</v>
       </c>
       <c r="H5" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="I5" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>221</v>
-      </c>
       <c r="K5" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L5" s="2">
         <v>8.5</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="N5" s="2">
         <v>80.53</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="P5" s="2">
         <v>1750</v>
@@ -2965,54 +2962,54 @@
         <v>9</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E6" s="2">
         <v>2778.33</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G6" s="2">
         <v>77.52</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="L6" s="2">
         <v>25</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="N6" s="2">
         <v>41.13</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="P6" s="2">
         <v>1400</v>
@@ -3027,54 +3024,54 @@
         <v>9</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="7" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E7" s="2">
         <v>5915.39</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G7" s="2">
         <v>60.14</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L7" s="2">
         <v>12</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="N7" s="2">
         <v>78.78</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="P7" s="2">
         <v>3000</v>
@@ -3089,54 +3086,54 @@
         <v>22</v>
       </c>
       <c r="T7" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="8" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E8" s="2">
         <v>1256.77</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G8" s="2">
         <v>92.17</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="L8" s="2">
         <v>180</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="N8" s="2">
         <v>84.76</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="P8" s="2">
         <v>600</v>
@@ -3151,54 +3148,54 @@
         <v>25</v>
       </c>
       <c r="T8" s="2" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E9" s="2">
         <v>1554.26</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G9" s="2">
         <v>71.09</v>
       </c>
       <c r="H9" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="J9" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="I9" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>214</v>
-      </c>
       <c r="K9" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L9" s="2">
         <v>18</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="N9" s="2">
         <v>74.680000000000007</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="P9" s="2">
         <v>750</v>
@@ -3213,54 +3210,54 @@
         <v>9</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E10" s="2">
         <v>3145.57</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G10" s="2">
         <v>82.54</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="L10" s="2">
         <v>35</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="N10" s="2">
         <v>51.68</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="P10" s="2">
         <v>1500</v>
@@ -3275,54 +3272,54 @@
         <v>15</v>
       </c>
       <c r="T10" s="2" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="11" spans="1:20" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E11" s="2">
         <v>789.19</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G11" s="2">
         <v>88.73</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="L11" s="2">
         <v>45</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="N11" s="2">
         <v>77.11</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="P11" s="2">
         <v>400</v>
@@ -3337,7 +3334,7 @@
         <v>15</v>
       </c>
       <c r="T11" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: recurring waste streams need a current batch
RC Interiors' plywood and OKA Basu's metal waste were marked Sold, so both
vanished from recommendations. That exclusion is right -- sold material
cannot be bought -- but the sheet records them as monthly production, 2,500
and 1,500 kg, not single consignments. The sold rows are history; what was
missing is this month's output.

Adding those batches also exposed a destructive key. Listings were matched on
plant and material alone, so a second batch from the same plant overwrote the
first -- and the first was the consignment RC Interiors sold to Al-Fas, the
one confirmed exchange in the dataset. The key now includes the availability
date, so a recurring stream keeps its history alongside its current stock.

Al-Fas searching for plywood now ranks RC Interiors first at 78.7%: 0.6 km
away, 98% quantity match, and the only candidate with a prior exchange. The
closed loop is visible in the product.
</commit_message>
<xml_diff>
--- a/datasets/kinfra_data.xlsx
+++ b/datasets/kinfra_data.xlsx
@@ -2889,7 +2889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T13"/>
+  <dimension ref="A1:T15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4069,6 +4069,182 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>KWST0013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>KM002</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>KP002</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>KC002</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>4920.6</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>84.09999999999999</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Indoor Storage</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>113.4</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>36.42</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>2026-09-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>2500</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>113.4</v>
+      </c>
+      <c r="R14" t="n">
+        <v>557996.04</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Sell as raw material</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Current batch of plywood offcuts and sawdust, about two months' output. Previous batch was sold to Al-Fas, who reprocess it into board.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>KWST0014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>KM009</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>KP009</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>KC009</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>3062.4</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>91.75</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Dry Storage</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>35</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>62.3</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>2026-09-11 00:00:00</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>1500</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>35</v>
+      </c>
+      <c r="R15" t="n">
+        <v>107184</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Sell to scrap dealer</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Current batch of steel and iron offcuts, about two months' output.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>